<commit_message>
n8n board refresh 2026-07-04T17:39:29Z
</commit_message>
<xml_diff>
--- a/app/reports/FNWD_research.xlsx
+++ b/app/reports/FNWD_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-03 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-04 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,7 @@
         <v>187380000</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>16.029629</v>
+        <v>15.79562</v>
       </c>
       <c r="E6" s="34" t="n"/>
       <c r="F6" s="34" t="n">
@@ -1567,7 +1567,7 @@
         <v>206899952</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>11.453238</v>
+        <v>11.494585</v>
       </c>
       <c r="E7" s="34" t="n"/>
       <c r="F7" s="34" t="n">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-07T17:39:54Z
</commit_message>
<xml_diff>
--- a/app/reports/FNWD_research.xlsx
+++ b/app/reports/FNWD_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-06 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-07 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.749</v>
+        <v>0.789</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>54.33</v>
+        <v>53.88</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>36.99</v>
+        <v>36.3</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.469</v>
+        <v>0.484</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.971</v>
+        <v>0.979</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.417</v>
+        <v>0.5</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.969</v>
+        <v>0.984</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04480999946594239</v>
+        <v>0.04525000095367432</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>4329971.127331711</v>
+        <v>4329970.688705235</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>36.99</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="38">
@@ -1520,14 +1520,14 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>160165632</v>
+        <v>157177936</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>16.15</v>
+        <v>15.85</v>
       </c>
       <c r="E5" s="32" t="n"/>
       <c r="F5" s="32" t="n">
-        <v>2.12</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="6">
@@ -1542,14 +1542,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>185561616</v>
+        <v>187726368</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>15.642336</v>
+        <v>16.05926</v>
       </c>
       <c r="E6" s="34" t="n"/>
       <c r="F6" s="34" t="n">
-        <v>3.214</v>
+        <v>3.185</v>
       </c>
     </row>
     <row r="7">
@@ -1564,14 +1564,14 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>206380096</v>
+        <v>207354816</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>11.465704</v>
+        <v>11.478417</v>
       </c>
       <c r="E7" s="34" t="n"/>
       <c r="F7" s="34" t="n">
-        <v>1.145</v>
+        <v>1.105</v>
       </c>
     </row>
     <row r="8">
@@ -1586,14 +1586,14 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>223743408</v>
+        <v>225141792</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>15.1634</v>
+        <v>15.25817</v>
       </c>
       <c r="E8" s="34" t="n"/>
       <c r="F8" s="34" t="n">
-        <v>5.859</v>
+        <v>5.758</v>
       </c>
     </row>
     <row r="9">
@@ -1608,14 +1608,14 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>175166944</v>
+        <v>175210704</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>17.25</v>
+        <v>17.25431</v>
       </c>
       <c r="E9" s="34" t="n"/>
       <c r="F9" s="34" t="n">
-        <v>9.067</v>
+        <v>9.052</v>
       </c>
     </row>
     <row r="10">
@@ -1630,14 +1630,14 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>215920576</v>
+        <v>210768448</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>12.363985</v>
+        <v>12.068966</v>
       </c>
       <c r="E10" s="34" t="n"/>
       <c r="F10" s="34" t="n">
-        <v>1.275</v>
+        <v>1.231</v>
       </c>
     </row>
     <row r="11">
@@ -1652,14 +1652,14 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>167465872</v>
+        <v>168897200</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>22.285715</v>
+        <v>22.476192</v>
       </c>
       <c r="E11" s="34" t="n"/>
       <c r="F11" s="34" t="n">
-        <v>1.659</v>
+        <v>1.652</v>
       </c>
     </row>
     <row r="12">
@@ -1674,14 +1674,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>191097280</v>
+        <v>188475328</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>10.012779</v>
+        <v>9.875399</v>
       </c>
       <c r="E12" s="34" t="n"/>
       <c r="F12" s="34" t="n">
-        <v>3.507</v>
+        <v>3.466</v>
       </c>
     </row>
     <row r="13">
@@ -1696,14 +1696,14 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>174474448</v>
+        <v>176645152</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>12.319095</v>
+        <v>12.472362</v>
       </c>
       <c r="E13" s="34" t="n"/>
       <c r="F13" s="34" t="n">
-        <v>1.325</v>
+        <v>1.326</v>
       </c>
     </row>
     <row r="15">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D17" s="36" t="n">
-        <v>0.667</v>
+        <v>0.5</v>
       </c>
       <c r="E17" s="36" t="n"/>
       <c r="F17" s="36" t="n">

</xml_diff>